<commit_message>
Añadidos comentarios en memético y modificados log en main
</commit_message>
<xml_diff>
--- a/material/Tablas_MH.xlsx
+++ b/material/Tablas_MH.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f05cc438dc355128/ANTIGUO/Documentos/PERSONAL/Universidad/Tercero/Primer_Cuatrimestre/Metaheuristicas/Practicas/practica2meta/material/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f05cc438dc355128/ANTIGUO/Documentos/PERSONAL/Universidad/Tercero/Primer_Cuatrimestre/Metaheuristicas/Practicas/practica3meta/material/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="109" documentId="13_ncr:1_{1EC32BA9-E4D7-4716-B5F6-9BC89E3DA072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75ECA646-EF7F-410B-8AEF-C586F83144F7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1467,7 +1467,7 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1491,8 +1491,8 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1501,6 +1501,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1517,11 +1520,20 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1530,29 +1542,17 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3184,6 +3184,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-B4B9-A64E-9C24-CF657EAA0927}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -3198,6 +3203,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-B4B9-A64E-9C24-CF657EAA0927}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -3529,6 +3539,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-3417-5645-8BDA-5742F54CEB11}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -3543,6 +3558,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-3417-5645-8BDA-5742F54CEB11}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -3557,6 +3577,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-3417-5645-8BDA-5742F54CEB11}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -8054,38 +8079,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA981"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.33203125" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" customWidth="1"/>
-    <col min="7" max="7" width="9.44140625" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.5" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.5" customWidth="1"/>
+    <col min="5" max="5" width="9.5" customWidth="1"/>
+    <col min="6" max="6" width="12.5" customWidth="1"/>
+    <col min="7" max="7" width="9.5" customWidth="1"/>
+    <col min="8" max="8" width="12.5" customWidth="1"/>
     <col min="9" max="9" width="13.33203125" customWidth="1"/>
-    <col min="10" max="26" width="10.44140625" customWidth="1"/>
+    <col min="10" max="26" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:26" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="41"/>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="105"/>
-      <c r="D1" s="104" t="s">
+      <c r="C1" s="107"/>
+      <c r="D1" s="106" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="105"/>
-      <c r="F1" s="104" t="s">
+      <c r="E1" s="107"/>
+      <c r="F1" s="106" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="105"/>
-      <c r="H1" s="104" t="s">
+      <c r="G1" s="107"/>
+      <c r="H1" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="105"/>
+      <c r="I1" s="107"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -8104,8 +8129,8 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="97" t="s">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A2" s="113" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -8150,30 +8175,30 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="98"/>
-      <c r="B3" s="100" t="s">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A3" s="85"/>
+      <c r="B3" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="102">
+      <c r="C3" s="110">
         <v>3542</v>
       </c>
-      <c r="D3" s="100" t="s">
+      <c r="D3" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="102">
+      <c r="E3" s="110">
         <v>26876</v>
       </c>
-      <c r="F3" s="100" t="s">
+      <c r="F3" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="102">
+      <c r="G3" s="110">
         <v>13292</v>
       </c>
-      <c r="H3" s="100" t="s">
+      <c r="H3" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="106">
+      <c r="I3" s="112">
         <v>150528</v>
       </c>
       <c r="J3" s="1"/>
@@ -8194,16 +8219,16 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="98"/>
-      <c r="B4" s="101"/>
-      <c r="C4" s="103"/>
-      <c r="D4" s="101"/>
-      <c r="E4" s="103"/>
-      <c r="F4" s="101"/>
-      <c r="G4" s="103"/>
-      <c r="H4" s="101"/>
-      <c r="I4" s="101"/>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A4" s="85"/>
+      <c r="B4" s="109"/>
+      <c r="C4" s="111"/>
+      <c r="D4" s="109"/>
+      <c r="E4" s="111"/>
+      <c r="F4" s="109"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="109"/>
+      <c r="I4" s="109"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -8222,8 +8247,8 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="99"/>
+    <row r="5" spans="1:26" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="86"/>
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -8266,7 +8291,7 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
@@ -8312,7 +8337,7 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>10</v>
       </c>
@@ -8349,8 +8374,8 @@
         <v>2.33888626098632E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2"/>
+    <row r="9" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="47"/>
       <c r="B9" s="38"/>
       <c r="C9" s="47"/>
@@ -8378,7 +8403,7 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:26" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="48" t="s">
         <v>21</v>
       </c>
@@ -8399,7 +8424,7 @@
       </c>
       <c r="I10" s="83"/>
     </row>
-    <row r="11" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="84" t="s">
         <v>20</v>
       </c>
@@ -8428,8 +8453,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="98"/>
+    <row r="12" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="85"/>
       <c r="B12" s="87" t="s">
         <v>6</v>
       </c>
@@ -8455,8 +8480,8 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="98"/>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A13" s="85"/>
       <c r="B13" s="88"/>
       <c r="C13" s="90"/>
       <c r="D13" s="88"/>
@@ -8466,8 +8491,8 @@
       <c r="H13" s="88"/>
       <c r="I13" s="90"/>
     </row>
-    <row r="14" spans="1:26" ht="17.399999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="99"/>
+    <row r="14" spans="1:26" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="86"/>
       <c r="B14" s="15" t="s">
         <v>7</v>
       </c>
@@ -8493,7 +8518,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:26" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="39" t="s">
         <v>11</v>
       </c>
@@ -8522,7 +8547,7 @@
         <v>7.8029999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="23" t="s">
         <v>12</v>
       </c>
@@ -8552,7 +8577,7 @@
       </c>
       <c r="J16" s="49"/>
     </row>
-    <row r="17" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
         <v>13</v>
       </c>
@@ -8581,7 +8606,7 @@
         <v>7.76</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
         <v>14</v>
       </c>
@@ -8610,7 +8635,7 @@
         <v>7.56</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
         <v>15</v>
       </c>
@@ -8639,7 +8664,7 @@
         <v>7.7434000000000003</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>10</v>
       </c>
@@ -8676,7 +8701,7 @@
         <v>7.7462799999999987</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
         <v>16</v>
       </c>
@@ -8713,7 +8738,7 @@
         <v>0.11424575265628059</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="37"/>
       <c r="B22" s="38"/>
       <c r="C22" s="38"/>
@@ -8724,7 +8749,7 @@
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
     </row>
-    <row r="23" spans="1:9" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:9" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="48" t="s">
         <v>22</v>
       </c>
@@ -8745,7 +8770,7 @@
       </c>
       <c r="I23" s="83"/>
     </row>
-    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="84" t="s">
         <v>20</v>
       </c>
@@ -8774,8 +8799,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="98"/>
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="85"/>
       <c r="B25" s="87" t="s">
         <v>6</v>
       </c>
@@ -8801,8 +8826,8 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="26" spans="1:9" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="98"/>
+    <row r="26" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="85"/>
       <c r="B26" s="88"/>
       <c r="C26" s="90"/>
       <c r="D26" s="88"/>
@@ -8812,8 +8837,8 @@
       <c r="H26" s="88"/>
       <c r="I26" s="90"/>
     </row>
-    <row r="27" spans="1:9" ht="17.399999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="99"/>
+    <row r="27" spans="1:9" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="86"/>
       <c r="B27" s="15" t="s">
         <v>7</v>
       </c>
@@ -8839,7 +8864,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
         <v>11</v>
       </c>
@@ -8868,7 +8893,7 @@
         <v>7.2930000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="23" t="s">
         <v>12</v>
       </c>
@@ -8897,7 +8922,7 @@
         <v>7.7889999999999997</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="23" t="s">
         <v>13</v>
       </c>
@@ -8926,7 +8951,7 @@
         <v>7.8970000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="23" t="s">
         <v>14</v>
       </c>
@@ -8955,7 +8980,7 @@
         <v>7.7629999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="24" t="s">
         <v>15</v>
       </c>
@@ -8984,7 +9009,7 @@
         <v>8.24</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
         <v>10</v>
       </c>
@@ -9021,7 +9046,7 @@
         <v>7.7964000000000002</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>16</v>
       </c>
@@ -9058,7 +9083,7 @@
         <v>0.33966277393909394</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="37"/>
       <c r="B35" s="38"/>
       <c r="C35" s="38"/>
@@ -9069,7 +9094,7 @@
       <c r="H35" s="38"/>
       <c r="I35" s="38"/>
     </row>
-    <row r="36" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="37"/>
       <c r="B36" s="38"/>
       <c r="C36" s="38"/>
@@ -9080,7 +9105,7 @@
       <c r="H36" s="38"/>
       <c r="I36" s="38"/>
     </row>
-    <row r="37" spans="1:9" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="37" spans="1:9" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="48" t="s">
         <v>23</v>
       </c>
@@ -9101,7 +9126,7 @@
       </c>
       <c r="I37" s="83"/>
     </row>
-    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="84" t="s">
         <v>20</v>
       </c>
@@ -9130,8 +9155,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="85"/>
+    <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="99"/>
       <c r="B39" s="87" t="s">
         <v>6</v>
       </c>
@@ -9157,8 +9182,8 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="40" spans="1:9" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="85"/>
+    <row r="40" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="99"/>
       <c r="B40" s="88"/>
       <c r="C40" s="90"/>
       <c r="D40" s="88"/>
@@ -9168,8 +9193,8 @@
       <c r="H40" s="88"/>
       <c r="I40" s="90"/>
     </row>
-    <row r="41" spans="1:9" ht="17.399999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="86"/>
+    <row r="41" spans="1:9" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="100"/>
       <c r="B41" s="15" t="s">
         <v>7</v>
       </c>
@@ -9195,7 +9220,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
         <v>11</v>
       </c>
@@ -9224,7 +9249,7 @@
         <v>7.3769999999999998</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="23" t="s">
         <v>12</v>
       </c>
@@ -9253,7 +9278,7 @@
         <v>7.8680000000000003</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="23" t="s">
         <v>13</v>
       </c>
@@ -9282,7 +9307,7 @@
         <v>7.43</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="23" t="s">
         <v>14</v>
       </c>
@@ -9311,7 +9336,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="24" t="s">
         <v>15</v>
       </c>
@@ -9340,7 +9365,7 @@
         <v>7.6239999999999997</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>10</v>
       </c>
@@ -9377,7 +9402,7 @@
         <v>7.5998000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>16</v>
       </c>
@@ -9414,29 +9439,29 @@
         <v>0.20064196968730172</v>
       </c>
     </row>
-    <row r="49" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" spans="1:15" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="49" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="50" spans="1:15" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="B50" s="91" t="s">
+      <c r="B50" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="C50" s="91"/>
-      <c r="D50" s="91" t="s">
+      <c r="C50" s="92"/>
+      <c r="D50" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="E50" s="91"/>
-      <c r="F50" s="91" t="s">
+      <c r="E50" s="92"/>
+      <c r="F50" s="92" t="s">
         <v>2</v>
       </c>
-      <c r="G50" s="91"/>
-      <c r="H50" s="91" t="s">
+      <c r="G50" s="92"/>
+      <c r="H50" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="I50" s="91"/>
-    </row>
-    <row r="51" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I50" s="92"/>
+    </row>
+    <row r="51" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="84" t="s">
         <v>20</v>
       </c>
@@ -9465,24 +9490,24 @@
         <v>30</v>
       </c>
     </row>
-    <row r="52" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="92"/>
+    <row r="52" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="93"/>
       <c r="B52" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="C52" s="95">
+      <c r="C52" s="96">
         <v>3542</v>
       </c>
       <c r="D52" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="E52" s="95">
+      <c r="E52" s="96">
         <v>26876</v>
       </c>
       <c r="F52" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="G52" s="95">
+      <c r="G52" s="96">
         <v>13292</v>
       </c>
       <c r="H52" s="87" t="s">
@@ -9492,19 +9517,19 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="92"/>
-      <c r="B53" s="94"/>
-      <c r="C53" s="96"/>
-      <c r="D53" s="94"/>
-      <c r="E53" s="96"/>
-      <c r="F53" s="94"/>
-      <c r="G53" s="96"/>
-      <c r="H53" s="94"/>
-      <c r="I53" s="107"/>
-    </row>
-    <row r="54" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="93"/>
+    <row r="53" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="93"/>
+      <c r="B53" s="95"/>
+      <c r="C53" s="97"/>
+      <c r="D53" s="95"/>
+      <c r="E53" s="97"/>
+      <c r="F53" s="95"/>
+      <c r="G53" s="97"/>
+      <c r="H53" s="95"/>
+      <c r="I53" s="98"/>
+    </row>
+    <row r="54" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="94"/>
       <c r="B54" s="15" t="s">
         <v>7</v>
       </c>
@@ -9534,7 +9559,7 @@
         <v>Media</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="22.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:15" ht="23" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="18" t="s">
         <v>11</v>
       </c>
@@ -9571,7 +9596,7 @@
         <v>0.13319249595987123</v>
       </c>
     </row>
-    <row r="56" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="23" t="s">
         <v>12</v>
       </c>
@@ -9608,7 +9633,7 @@
         <v>9.3057275778411996E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="23" t="s">
         <v>13</v>
       </c>
@@ -9645,7 +9670,7 @@
         <v>0.10122557602816315</v>
       </c>
     </row>
-    <row r="58" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="23" t="s">
         <v>14</v>
       </c>
@@ -9682,7 +9707,7 @@
         <v>8.2873045156951458E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="24" t="s">
         <v>15</v>
       </c>
@@ -9711,7 +9736,7 @@
         <v>7.8129999999999997</v>
       </c>
     </row>
-    <row r="60" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>10</v>
       </c>
@@ -9748,7 +9773,7 @@
         <v>7.9346000000000005</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23" t="s">
         <v>16</v>
       </c>
@@ -9785,13 +9810,13 @@
         <v>0.24113440235686009</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="67" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="75" t="s">
+    <row r="62" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="63" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="64" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="65" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="66" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="91" t="s">
         <v>33</v>
       </c>
       <c r="B67" s="76" t="s">
@@ -9815,8 +9840,8 @@
       </c>
       <c r="K67" s="81"/>
     </row>
-    <row r="68" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="75"/>
+    <row r="68" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="91"/>
       <c r="B68" s="15" t="s">
         <v>10</v>
       </c>
@@ -9848,7 +9873,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="69" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="55" t="s">
         <v>38</v>
       </c>
@@ -9893,7 +9918,7 @@
         <v>5.7770200000000003</v>
       </c>
     </row>
-    <row r="70" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A70" s="54" t="s">
         <v>39</v>
       </c>
@@ -9938,7 +9963,7 @@
         <v>5.8417499999999993</v>
       </c>
     </row>
-    <row r="71" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A71" s="54" t="s">
         <v>40</v>
       </c>
@@ -9983,7 +10008,7 @@
         <v>5.7248000000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:27" ht="58.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:27" ht="66" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="54" t="s">
         <v>41</v>
       </c>
@@ -10039,7 +10064,7 @@
         <v>5.9914999999999994</v>
       </c>
     </row>
-    <row r="73" spans="1:27" ht="61.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:27" ht="68" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A73" s="30"/>
       <c r="Y73" s="54" t="s">
         <v>37</v>
@@ -10053,10 +10078,10 @@
         <v>5.8832500000000003</v>
       </c>
     </row>
-    <row r="74" spans="1:27" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="75" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="76" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="75" t="s">
+    <row r="74" spans="1:27" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="75" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="91" t="s">
         <v>33</v>
       </c>
       <c r="B76" s="76" t="s">
@@ -10080,8 +10105,8 @@
       </c>
       <c r="K76" s="81"/>
     </row>
-    <row r="77" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="75"/>
+    <row r="77" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="91"/>
       <c r="B77" s="15" t="s">
         <v>18</v>
       </c>
@@ -10113,7 +10138,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="78" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="55" t="s">
         <v>38</v>
       </c>
@@ -10158,7 +10183,7 @@
         <v>0.20623427122159527</v>
       </c>
     </row>
-    <row r="79" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A79" s="54" t="s">
         <v>39</v>
       </c>
@@ -10203,7 +10228,7 @@
         <v>0.2904571327202502</v>
       </c>
     </row>
-    <row r="80" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="54" t="s">
         <v>40</v>
       </c>
@@ -10248,7 +10273,7 @@
         <v>0.17863270933809342</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A81" s="54" t="s">
         <v>41</v>
       </c>
@@ -10293,35 +10318,35 @@
         <v>0.17365208089750223</v>
       </c>
     </row>
-    <row r="82" spans="1:11" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="83" spans="1:11" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.7">
+    <row r="82" spans="1:11" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="83" spans="1:11" ht="36" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A83" s="56" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="84" spans="1:11" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A84" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="B84" s="108" t="s">
+      <c r="B84" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="C84" s="109"/>
-      <c r="D84" s="108" t="s">
+      <c r="C84" s="104"/>
+      <c r="D84" s="103" t="s">
         <v>1</v>
       </c>
-      <c r="E84" s="109"/>
-      <c r="F84" s="108" t="s">
+      <c r="E84" s="104"/>
+      <c r="F84" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="G84" s="109"/>
-      <c r="H84" s="108" t="s">
+      <c r="G84" s="104"/>
+      <c r="H84" s="103" t="s">
         <v>3</v>
       </c>
-      <c r="I84" s="110"/>
-    </row>
-    <row r="85" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="111" t="s">
+      <c r="I84" s="105"/>
+    </row>
+    <row r="85" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="114" t="s">
         <v>20</v>
       </c>
       <c r="B85" s="12" t="s">
@@ -10349,8 +10374,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="112"/>
+    <row r="86" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="115"/>
       <c r="B86" s="87" t="s">
         <v>6</v>
       </c>
@@ -10372,12 +10397,12 @@
       <c r="H86" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="I86" s="114">
+      <c r="I86" s="101">
         <v>150528</v>
       </c>
     </row>
-    <row r="87" spans="1:11" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A87" s="112"/>
+    <row r="87" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="115"/>
       <c r="B87" s="88"/>
       <c r="C87" s="90"/>
       <c r="D87" s="88"/>
@@ -10385,10 +10410,10 @@
       <c r="F87" s="88"/>
       <c r="G87" s="90"/>
       <c r="H87" s="88"/>
-      <c r="I87" s="115"/>
-    </row>
-    <row r="88" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A88" s="113"/>
+      <c r="I87" s="102"/>
+    </row>
+    <row r="88" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="116"/>
       <c r="B88" s="60" t="s">
         <v>7</v>
       </c>
@@ -10414,7 +10439,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A89" s="62" t="s">
         <v>11</v>
       </c>
@@ -10443,7 +10468,7 @@
         <v>9.4290000000000003</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A90" s="65" t="s">
         <v>12</v>
       </c>
@@ -10473,7 +10498,7 @@
       </c>
       <c r="J90" s="49"/>
     </row>
-    <row r="91" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A91" s="65" t="s">
         <v>13</v>
       </c>
@@ -10502,7 +10527,7 @@
         <v>7.91</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A92" s="65" t="s">
         <v>14</v>
       </c>
@@ -10531,7 +10556,7 @@
         <v>7.7910000000000004</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A93" s="66" t="s">
         <v>15</v>
       </c>
@@ -10560,7 +10585,7 @@
         <v>7.8465999999999996</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A94" s="68" t="s">
         <v>10</v>
       </c>
@@ -10597,7 +10622,7 @@
         <v>8.1249199999999995</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A95" s="70" t="s">
         <v>16</v>
       </c>
@@ -10634,7 +10659,7 @@
         <v>0.73539658144432529</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="37"/>
       <c r="B96" s="38"/>
       <c r="C96" s="38"/>
@@ -10645,7 +10670,7 @@
       <c r="H96" s="38"/>
       <c r="I96" s="38"/>
     </row>
-    <row r="97" spans="1:9" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="97" spans="1:9" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A97" s="48" t="s">
         <v>27</v>
       </c>
@@ -10666,7 +10691,7 @@
       </c>
       <c r="I97" s="83"/>
     </row>
-    <row r="98" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="84" t="s">
         <v>20</v>
       </c>
@@ -10695,8 +10720,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="98"/>
+    <row r="99" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="85"/>
       <c r="B99" s="87" t="s">
         <v>6</v>
       </c>
@@ -10722,8 +10747,8 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A100" s="98"/>
+    <row r="100" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="85"/>
       <c r="B100" s="88"/>
       <c r="C100" s="90"/>
       <c r="D100" s="88"/>
@@ -10733,8 +10758,8 @@
       <c r="H100" s="88"/>
       <c r="I100" s="90"/>
     </row>
-    <row r="101" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="99"/>
+    <row r="101" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="86"/>
       <c r="B101" s="15" t="s">
         <v>7</v>
       </c>
@@ -10760,7 +10785,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A102" s="39" t="s">
         <v>11</v>
       </c>
@@ -10789,7 +10814,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A103" s="23" t="s">
         <v>12</v>
       </c>
@@ -10818,7 +10843,7 @@
         <v>7.63</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A104" s="23" t="s">
         <v>13</v>
       </c>
@@ -10847,7 +10872,7 @@
         <v>8.07</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A105" s="23" t="s">
         <v>14</v>
       </c>
@@ -10876,7 +10901,7 @@
         <v>7.38</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A106" s="24" t="s">
         <v>15</v>
       </c>
@@ -10905,7 +10930,7 @@
         <v>7.69</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A107" s="9" t="s">
         <v>10</v>
       </c>
@@ -10942,7 +10967,7 @@
         <v>7.6340000000000003</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A108" s="23" t="s">
         <v>16</v>
       </c>
@@ -10979,7 +11004,7 @@
         <v>0.27951744131628004</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="37"/>
       <c r="B109" s="38"/>
       <c r="C109" s="38"/>
@@ -10990,7 +11015,7 @@
       <c r="H109" s="38"/>
       <c r="I109" s="38"/>
     </row>
-    <row r="110" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="37"/>
       <c r="B110" s="38"/>
       <c r="C110" s="38"/>
@@ -11001,7 +11026,7 @@
       <c r="H110" s="38"/>
       <c r="I110" s="38"/>
     </row>
-    <row r="111" spans="1:9" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="111" spans="1:9" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A111" s="48" t="s">
         <v>28</v>
       </c>
@@ -11022,7 +11047,7 @@
       </c>
       <c r="I111" s="83"/>
     </row>
-    <row r="112" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="84" t="s">
         <v>20</v>
       </c>
@@ -11051,8 +11076,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="85"/>
+    <row r="113" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="99"/>
       <c r="B113" s="87" t="s">
         <v>6</v>
       </c>
@@ -11078,8 +11103,8 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="85"/>
+    <row r="114" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="99"/>
       <c r="B114" s="88"/>
       <c r="C114" s="90"/>
       <c r="D114" s="88"/>
@@ -11089,8 +11114,8 @@
       <c r="H114" s="88"/>
       <c r="I114" s="90"/>
     </row>
-    <row r="115" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A115" s="86"/>
+    <row r="115" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="100"/>
       <c r="B115" s="15" t="s">
         <v>7</v>
       </c>
@@ -11116,7 +11141,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A116" s="18" t="s">
         <v>11</v>
       </c>
@@ -11154,7 +11179,7 @@
       <c r="Q116" s="49"/>
       <c r="R116" s="57"/>
     </row>
-    <row r="117" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A117" s="23" t="s">
         <v>12</v>
       </c>
@@ -11192,7 +11217,7 @@
       <c r="Q117" s="57"/>
       <c r="R117" s="57"/>
     </row>
-    <row r="118" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A118" s="23" t="s">
         <v>13</v>
       </c>
@@ -11221,7 +11246,7 @@
         <v>7.73</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
         <v>14</v>
       </c>
@@ -11250,7 +11275,7 @@
         <v>7.84</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24" t="s">
         <v>15</v>
       </c>
@@ -11279,7 +11304,7 @@
         <v>7.8959999999999999</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A121" s="9" t="s">
         <v>10</v>
       </c>
@@ -11316,7 +11341,7 @@
         <v>7.7471999999999994</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A122" s="23" t="s">
         <v>16</v>
       </c>
@@ -11353,29 +11378,29 @@
         <v>0.14376786845467254</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="124" spans="1:18" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="123" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="124" spans="1:18" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A124" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="B124" s="91" t="s">
+      <c r="B124" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="C124" s="91"/>
-      <c r="D124" s="91" t="s">
+      <c r="C124" s="92"/>
+      <c r="D124" s="92" t="s">
         <v>1</v>
       </c>
-      <c r="E124" s="91"/>
-      <c r="F124" s="91" t="s">
+      <c r="E124" s="92"/>
+      <c r="F124" s="92" t="s">
         <v>2</v>
       </c>
-      <c r="G124" s="91"/>
-      <c r="H124" s="91" t="s">
+      <c r="G124" s="92"/>
+      <c r="H124" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="I124" s="91"/>
-    </row>
-    <row r="125" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I124" s="92"/>
+    </row>
+    <row r="125" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="84" t="s">
         <v>20</v>
       </c>
@@ -11404,24 +11429,24 @@
         <v>30</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="92"/>
+    <row r="126" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A126" s="93"/>
       <c r="B126" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="C126" s="95">
+      <c r="C126" s="96">
         <v>3542</v>
       </c>
       <c r="D126" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="E126" s="95">
+      <c r="E126" s="96">
         <v>26876</v>
       </c>
       <c r="F126" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="G126" s="95">
+      <c r="G126" s="96">
         <v>13292</v>
       </c>
       <c r="H126" s="87" t="s">
@@ -11431,19 +11456,19 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="127" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A127" s="92"/>
-      <c r="B127" s="94"/>
-      <c r="C127" s="96"/>
-      <c r="D127" s="94"/>
-      <c r="E127" s="96"/>
-      <c r="F127" s="94"/>
-      <c r="G127" s="96"/>
-      <c r="H127" s="94"/>
-      <c r="I127" s="107"/>
-    </row>
-    <row r="128" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A128" s="93"/>
+    <row r="127" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="93"/>
+      <c r="B127" s="95"/>
+      <c r="C127" s="97"/>
+      <c r="D127" s="95"/>
+      <c r="E127" s="97"/>
+      <c r="F127" s="95"/>
+      <c r="G127" s="97"/>
+      <c r="H127" s="95"/>
+      <c r="I127" s="98"/>
+    </row>
+    <row r="128" spans="1:18" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="94"/>
       <c r="B128" s="15" t="s">
         <v>7</v>
       </c>
@@ -11473,7 +11498,7 @@
         <v>Media</v>
       </c>
     </row>
-    <row r="129" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A129" s="18" t="s">
         <v>11</v>
       </c>
@@ -11510,7 +11535,7 @@
         <v>0.12882639687990155</v>
       </c>
     </row>
-    <row r="130" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A130" s="23" t="s">
         <v>12</v>
       </c>
@@ -11547,7 +11572,7 @@
         <v>9.1616172235781168E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A131" s="23" t="s">
         <v>13</v>
       </c>
@@ -11584,7 +11609,7 @@
         <v>9.3756936043993627E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A132" s="23" t="s">
         <v>14</v>
       </c>
@@ -11621,7 +11646,7 @@
         <v>7.2317833124453404E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A133" s="24" t="s">
         <v>15</v>
       </c>
@@ -11650,7 +11675,7 @@
         <v>7.83</v>
       </c>
     </row>
-    <row r="134" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A134" s="9" t="s">
         <v>10</v>
       </c>
@@ -11687,7 +11712,7 @@
         <v>7.8109999999999999</v>
       </c>
     </row>
-    <row r="135" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A135" s="23" t="s">
         <v>16</v>
       </c>
@@ -11724,13 +11749,13 @@
         <v>6.8044103344816032E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="137" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="138" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="139" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="140" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="141" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A141" s="75" t="s">
+    <row r="136" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="137" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="138" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="139" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="140" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="91" t="s">
         <v>25</v>
       </c>
       <c r="B141" s="76" t="s">
@@ -11754,8 +11779,8 @@
       </c>
       <c r="K141" s="81"/>
     </row>
-    <row r="142" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A142" s="75"/>
+    <row r="142" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="91"/>
       <c r="B142" s="15" t="s">
         <v>10</v>
       </c>
@@ -11787,7 +11812,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="143" spans="1:15" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:15" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A143" s="54" t="s">
         <v>34</v>
       </c>
@@ -11832,7 +11857,7 @@
         <v>5.9780599999999993</v>
       </c>
     </row>
-    <row r="144" spans="1:15" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:15" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A144" s="54" t="s">
         <v>35</v>
       </c>
@@ -11877,7 +11902,7 @@
         <v>5.7455499999999997</v>
       </c>
     </row>
-    <row r="145" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A145" s="54" t="s">
         <v>36</v>
       </c>
@@ -11922,7 +11947,7 @@
         <v>5.8456000000000001</v>
       </c>
     </row>
-    <row r="146" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A146" s="54" t="s">
         <v>37</v>
       </c>
@@ -11967,13 +11992,13 @@
         <v>5.8832500000000003</v>
       </c>
     </row>
-    <row r="147" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
+    <row r="147" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A147" s="30"/>
     </row>
-    <row r="148" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="149" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="150" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A150" s="75" t="s">
+    <row r="148" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="149" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="91" t="s">
         <v>25</v>
       </c>
       <c r="B150" s="76" t="s">
@@ -11997,8 +12022,8 @@
       </c>
       <c r="K150" s="81"/>
     </row>
-    <row r="151" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A151" s="75"/>
+    <row r="151" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="91"/>
       <c r="B151" s="15" t="s">
         <v>18</v>
       </c>
@@ -12030,7 +12055,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="152" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A152" s="54" t="s">
         <v>34</v>
       </c>
@@ -12075,7 +12100,7 @@
         <v>0.46866537961257426</v>
       </c>
     </row>
-    <row r="153" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A153" s="54" t="s">
         <v>35</v>
       </c>
@@ -12120,7 +12145,7 @@
         <v>0.20640440657776393</v>
       </c>
     </row>
-    <row r="154" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A154" s="54" t="s">
         <v>36</v>
       </c>
@@ -12165,7 +12190,7 @@
         <v>0.11924920614065483</v>
       </c>
     </row>
-    <row r="155" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A155" s="54" t="s">
         <v>37</v>
       </c>
@@ -12210,15 +12235,15 @@
         <v>0.14856237750823093</v>
       </c>
     </row>
-    <row r="156" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="157" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="158" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="159" spans="1:11" ht="67.2" x14ac:dyDescent="0.65">
+    <row r="156" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="157" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="158" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="159" spans="1:11" ht="70" x14ac:dyDescent="0.4">
       <c r="A159" s="56" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="160" spans="1:11" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="160" spans="1:11" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A160" s="48" t="s">
         <v>31</v>
       </c>
@@ -12239,7 +12264,7 @@
       </c>
       <c r="I160" s="83"/>
     </row>
-    <row r="161" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="84" t="s">
         <v>30</v>
       </c>
@@ -12268,8 +12293,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="162" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="98"/>
+    <row r="162" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" s="85"/>
       <c r="B162" s="87" t="s">
         <v>6</v>
       </c>
@@ -12295,8 +12320,8 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="163" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A163" s="98"/>
+    <row r="163" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="85"/>
       <c r="B163" s="88"/>
       <c r="C163" s="90"/>
       <c r="D163" s="88"/>
@@ -12306,8 +12331,8 @@
       <c r="H163" s="88"/>
       <c r="I163" s="90"/>
     </row>
-    <row r="164" spans="1:10" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A164" s="99"/>
+    <row r="164" spans="1:10" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="86"/>
       <c r="B164" s="15" t="s">
         <v>7</v>
       </c>
@@ -12333,7 +12358,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A165" s="39" t="s">
         <v>11</v>
       </c>
@@ -12362,7 +12387,7 @@
         <v>19.41</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A166" s="23" t="s">
         <v>12</v>
       </c>
@@ -12392,7 +12417,7 @@
       </c>
       <c r="J166" s="49"/>
     </row>
-    <row r="167" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A167" s="23" t="s">
         <v>13</v>
       </c>
@@ -12421,7 +12446,7 @@
         <v>32.25</v>
       </c>
     </row>
-    <row r="168" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A168" s="23" t="s">
         <v>14</v>
       </c>
@@ -12450,7 +12475,7 @@
         <v>30.67</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A169" s="24" t="s">
         <v>15</v>
       </c>
@@ -12479,7 +12504,7 @@
         <v>31.02</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A170" s="9" t="s">
         <v>10</v>
       </c>
@@ -12516,7 +12541,7 @@
         <v>28.887999999999998</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A171" s="23" t="s">
         <v>16</v>
       </c>
@@ -12553,7 +12578,7 @@
         <v>5.3316338959084399</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="37"/>
       <c r="B172" s="38"/>
       <c r="C172" s="38"/>
@@ -12564,7 +12589,7 @@
       <c r="H172" s="38"/>
       <c r="I172" s="38"/>
     </row>
-    <row r="173" spans="1:10" ht="31.2" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="173" spans="1:10" ht="35" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A173" s="48" t="s">
         <v>32</v>
       </c>
@@ -12585,7 +12610,7 @@
       </c>
       <c r="I173" s="83"/>
     </row>
-    <row r="174" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="84" t="s">
         <v>30</v>
       </c>
@@ -12614,8 +12639,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A175" s="98"/>
+    <row r="175" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" s="85"/>
       <c r="B175" s="87" t="s">
         <v>6</v>
       </c>
@@ -12641,8 +12666,8 @@
         <v>150528</v>
       </c>
     </row>
-    <row r="176" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A176" s="98"/>
+    <row r="176" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="85"/>
       <c r="B176" s="88"/>
       <c r="C176" s="90"/>
       <c r="D176" s="88"/>
@@ -12652,8 +12677,8 @@
       <c r="H176" s="88"/>
       <c r="I176" s="90"/>
     </row>
-    <row r="177" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A177" s="99"/>
+    <row r="177" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="86"/>
       <c r="B177" s="15" t="s">
         <v>7</v>
       </c>
@@ -12679,7 +12704,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="178" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A178" s="39" t="s">
         <v>11</v>
       </c>
@@ -12708,7 +12733,7 @@
         <v>29.26</v>
       </c>
     </row>
-    <row r="179" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A179" s="23" t="s">
         <v>12</v>
       </c>
@@ -12737,7 +12762,7 @@
         <v>29.32</v>
       </c>
     </row>
-    <row r="180" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A180" s="23" t="s">
         <v>13</v>
       </c>
@@ -12766,7 +12791,7 @@
         <v>31.344000000000001</v>
       </c>
     </row>
-    <row r="181" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A181" s="23" t="s">
         <v>14</v>
       </c>
@@ -12795,7 +12820,7 @@
         <v>31.11</v>
       </c>
     </row>
-    <row r="182" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A182" s="24" t="s">
         <v>15</v>
       </c>
@@ -12824,7 +12849,7 @@
         <v>31.35</v>
       </c>
     </row>
-    <row r="183" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A183" s="9" t="s">
         <v>10</v>
       </c>
@@ -12861,7 +12886,7 @@
         <v>30.476800000000004</v>
       </c>
     </row>
-    <row r="184" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A184" s="23" t="s">
         <v>16</v>
       </c>
@@ -12898,7 +12923,7 @@
         <v>1.0879159894035937</v>
       </c>
     </row>
-    <row r="185" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="37"/>
       <c r="B185" s="38"/>
       <c r="C185" s="38"/>
@@ -12909,11 +12934,11 @@
       <c r="H185" s="38"/>
       <c r="I185" s="38"/>
     </row>
-    <row r="186" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="187" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="188" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="189" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A189" s="116"/>
+    <row r="186" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="187" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="188" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="1:15" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="75"/>
       <c r="B189" s="76" t="s">
         <v>0</v>
       </c>
@@ -12939,8 +12964,8 @@
         <v>Media</v>
       </c>
     </row>
-    <row r="190" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A190" s="116"/>
+    <row r="190" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="75"/>
       <c r="B190" s="15" t="s">
         <v>10</v>
       </c>
@@ -12980,7 +13005,7 @@
         <v>0.12737465087623068</v>
       </c>
     </row>
-    <row r="191" spans="1:15" ht="94.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:15" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A191" s="54" t="s">
         <v>31</v>
       </c>
@@ -13033,7 +13058,7 @@
         <v>0.10663714037406641</v>
       </c>
     </row>
-    <row r="192" spans="1:15" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:15" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A192" s="54" t="s">
         <v>32</v>
       </c>
@@ -13080,10 +13105,10 @@
       <c r="N192" s="40"/>
       <c r="O192" s="42"/>
     </row>
-    <row r="193" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="194" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="195" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A195" s="116"/>
+    <row r="193" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="194" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="75"/>
       <c r="B195" s="76" t="s">
         <v>0</v>
       </c>
@@ -13105,8 +13130,8 @@
       </c>
       <c r="K195" s="81"/>
     </row>
-    <row r="196" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A196" s="116"/>
+    <row r="196" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="75"/>
       <c r="B196" s="15" t="s">
         <v>18</v>
       </c>
@@ -13138,7 +13163,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="197" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A197" s="54" t="s">
         <v>31</v>
       </c>
@@ -13183,7 +13208,7 @@
         <v>2.8415528327647808</v>
       </c>
     </row>
-    <row r="198" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A198" s="54" t="s">
         <v>32</v>
       </c>
@@ -13228,16 +13253,16 @@
         <v>1.9920843141337421</v>
       </c>
     </row>
-    <row r="199" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="200" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="201" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="200" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="201" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" s="74" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="202" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="203" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A203" s="116"/>
+    <row r="202" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="1:11" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A203" s="75"/>
       <c r="B203" s="76" t="s">
         <v>0</v>
       </c>
@@ -13259,8 +13284,8 @@
       </c>
       <c r="K203" s="81"/>
     </row>
-    <row r="204" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A204" s="116"/>
+    <row r="204" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="75"/>
       <c r="B204" s="15" t="s">
         <v>18</v>
       </c>
@@ -13292,7 +13317,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="205" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A205" s="54" t="s">
         <v>41</v>
       </c>
@@ -13327,7 +13352,7 @@
         <v>0.17365208089750223</v>
       </c>
     </row>
-    <row r="206" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:11" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A206" s="54" t="s">
         <v>37</v>
       </c>
@@ -13362,16 +13387,16 @@
         <v>0.14856237750823093</v>
       </c>
     </row>
-    <row r="207" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="208" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="209" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="208" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="209" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="74" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="210" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="211" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A211" s="75" t="s">
+    <row r="210" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="91" t="s">
         <v>43</v>
       </c>
       <c r="B211" s="76" t="s">
@@ -13395,8 +13420,8 @@
       </c>
       <c r="K211" s="81"/>
     </row>
-    <row r="212" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A212" s="75"/>
+    <row r="212" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A212" s="91"/>
       <c r="B212" s="15" t="s">
         <v>10</v>
       </c>
@@ -13443,7 +13468,7 @@
         <v>5.8832500000000003</v>
       </c>
     </row>
-    <row r="213" spans="1:27" ht="87.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:27" ht="82" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A213" s="54" t="s">
         <v>46</v>
       </c>
@@ -13493,7 +13518,7 @@
         <v>27.933700000000002</v>
       </c>
     </row>
-    <row r="214" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A214" s="54" t="s">
         <v>45</v>
       </c>
@@ -13543,7 +13568,7 @@
         <v>38.497052233219122</v>
       </c>
     </row>
-    <row r="215" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A215" s="54" t="s">
         <v>44</v>
       </c>
@@ -13578,10 +13603,10 @@
         <v>38.497052233219122</v>
       </c>
     </row>
-    <row r="216" spans="1:27" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="217" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="218" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A218" s="116"/>
+    <row r="216" spans="1:27" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="217" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="75"/>
       <c r="B218" s="76" t="s">
         <v>0</v>
       </c>
@@ -13603,8 +13628,8 @@
       </c>
       <c r="K218" s="81"/>
     </row>
-    <row r="219" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A219" s="116"/>
+    <row r="219" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="75"/>
       <c r="B219" s="15" t="s">
         <v>18</v>
       </c>
@@ -13636,7 +13661,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="220" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A220" s="54" t="s">
         <v>46</v>
       </c>
@@ -13671,7 +13696,7 @@
         <v>0.14856237750823093</v>
       </c>
     </row>
-    <row r="221" spans="1:27" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:27" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A221" s="54" t="s">
         <v>45</v>
       </c>
@@ -13716,7 +13741,7 @@
         <v>1.9920843141337421</v>
       </c>
     </row>
-    <row r="222" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:27" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A222" s="54" t="s">
         <v>44</v>
       </c>
@@ -13751,904 +13776,791 @@
         <v>0.75069407907573382</v>
       </c>
     </row>
-    <row r="223" spans="1:27" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="224" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="223" spans="1:27" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="224" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="197">
-    <mergeCell ref="A218:A219"/>
-    <mergeCell ref="B218:C218"/>
-    <mergeCell ref="D218:E218"/>
-    <mergeCell ref="F218:G218"/>
-    <mergeCell ref="H218:I218"/>
-    <mergeCell ref="J218:K218"/>
-    <mergeCell ref="A203:A204"/>
-    <mergeCell ref="B203:C203"/>
-    <mergeCell ref="D203:E203"/>
-    <mergeCell ref="F203:G203"/>
-    <mergeCell ref="H203:I203"/>
-    <mergeCell ref="J203:K203"/>
-    <mergeCell ref="J189:K189"/>
-    <mergeCell ref="A195:A196"/>
-    <mergeCell ref="B195:C195"/>
-    <mergeCell ref="D195:E195"/>
-    <mergeCell ref="F195:G195"/>
-    <mergeCell ref="H195:I195"/>
-    <mergeCell ref="J195:K195"/>
-    <mergeCell ref="A189:A190"/>
-    <mergeCell ref="B189:C189"/>
-    <mergeCell ref="D189:E189"/>
-    <mergeCell ref="F189:G189"/>
-    <mergeCell ref="H189:I189"/>
-    <mergeCell ref="B173:C173"/>
-    <mergeCell ref="D173:E173"/>
-    <mergeCell ref="F173:G173"/>
-    <mergeCell ref="H173:I173"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="B175:B176"/>
-    <mergeCell ref="C175:C176"/>
-    <mergeCell ref="D175:D176"/>
-    <mergeCell ref="E175:E176"/>
-    <mergeCell ref="F175:F176"/>
-    <mergeCell ref="G175:G176"/>
-    <mergeCell ref="H175:H176"/>
-    <mergeCell ref="I175:I176"/>
-    <mergeCell ref="B160:C160"/>
-    <mergeCell ref="D160:E160"/>
-    <mergeCell ref="F160:G160"/>
-    <mergeCell ref="H160:I160"/>
-    <mergeCell ref="A161:A164"/>
-    <mergeCell ref="B162:B163"/>
-    <mergeCell ref="C162:C163"/>
-    <mergeCell ref="D162:D163"/>
-    <mergeCell ref="E162:E163"/>
-    <mergeCell ref="F162:F163"/>
-    <mergeCell ref="G162:G163"/>
-    <mergeCell ref="H162:H163"/>
-    <mergeCell ref="I162:I163"/>
-    <mergeCell ref="J141:K141"/>
-    <mergeCell ref="A150:A151"/>
-    <mergeCell ref="B150:C150"/>
-    <mergeCell ref="D150:E150"/>
-    <mergeCell ref="F150:G150"/>
-    <mergeCell ref="H150:I150"/>
-    <mergeCell ref="J150:K150"/>
-    <mergeCell ref="A141:A142"/>
-    <mergeCell ref="B141:C141"/>
-    <mergeCell ref="D141:E141"/>
-    <mergeCell ref="F141:G141"/>
-    <mergeCell ref="H141:I141"/>
-    <mergeCell ref="B124:C124"/>
-    <mergeCell ref="D124:E124"/>
-    <mergeCell ref="F124:G124"/>
-    <mergeCell ref="H124:I124"/>
-    <mergeCell ref="A125:A128"/>
-    <mergeCell ref="B126:B127"/>
-    <mergeCell ref="C126:C127"/>
-    <mergeCell ref="D126:D127"/>
-    <mergeCell ref="E126:E127"/>
-    <mergeCell ref="F126:F127"/>
-    <mergeCell ref="G126:G127"/>
-    <mergeCell ref="H126:H127"/>
-    <mergeCell ref="I126:I127"/>
-    <mergeCell ref="B111:C111"/>
-    <mergeCell ref="D111:E111"/>
-    <mergeCell ref="F111:G111"/>
-    <mergeCell ref="H111:I111"/>
-    <mergeCell ref="A112:A115"/>
-    <mergeCell ref="B113:B114"/>
-    <mergeCell ref="C113:C114"/>
-    <mergeCell ref="D113:D114"/>
-    <mergeCell ref="E113:E114"/>
-    <mergeCell ref="F113:F114"/>
-    <mergeCell ref="G113:G114"/>
-    <mergeCell ref="H113:H114"/>
-    <mergeCell ref="I113:I114"/>
-    <mergeCell ref="G86:G87"/>
-    <mergeCell ref="H86:H87"/>
-    <mergeCell ref="I86:I87"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="D97:E97"/>
-    <mergeCell ref="F97:G97"/>
-    <mergeCell ref="H97:I97"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="B99:B100"/>
-    <mergeCell ref="C99:C100"/>
-    <mergeCell ref="D99:D100"/>
-    <mergeCell ref="E99:E100"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G99:G100"/>
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="I99:I100"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="H52:H53"/>
-    <mergeCell ref="I52:I53"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="D84:E84"/>
-    <mergeCell ref="F84:G84"/>
-    <mergeCell ref="H84:I84"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J67:K67"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="H67:I67"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="J76:K76"/>
+    <mergeCell ref="A76:A77"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="D37:E37"/>
     <mergeCell ref="B50:C50"/>
     <mergeCell ref="D50:E50"/>
     <mergeCell ref="F50:G50"/>
@@ -14673,42 +14585,155 @@
     <mergeCell ref="E12:E13"/>
     <mergeCell ref="F12:F13"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="H39:H40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="G52:G53"/>
+    <mergeCell ref="H52:H53"/>
+    <mergeCell ref="I52:I53"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="D84:E84"/>
+    <mergeCell ref="F84:G84"/>
+    <mergeCell ref="H84:I84"/>
+    <mergeCell ref="G86:G87"/>
+    <mergeCell ref="H86:H87"/>
+    <mergeCell ref="I86:I87"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="D97:E97"/>
+    <mergeCell ref="F97:G97"/>
+    <mergeCell ref="H97:I97"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B99:B100"/>
+    <mergeCell ref="C99:C100"/>
+    <mergeCell ref="D99:D100"/>
+    <mergeCell ref="E99:E100"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G99:G100"/>
+    <mergeCell ref="H99:H100"/>
+    <mergeCell ref="I99:I100"/>
+    <mergeCell ref="A85:A88"/>
+    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="C86:C87"/>
+    <mergeCell ref="D86:D87"/>
+    <mergeCell ref="E86:E87"/>
+    <mergeCell ref="F86:F87"/>
+    <mergeCell ref="B111:C111"/>
+    <mergeCell ref="D111:E111"/>
+    <mergeCell ref="F111:G111"/>
+    <mergeCell ref="H111:I111"/>
+    <mergeCell ref="A112:A115"/>
+    <mergeCell ref="B113:B114"/>
+    <mergeCell ref="C113:C114"/>
+    <mergeCell ref="D113:D114"/>
+    <mergeCell ref="E113:E114"/>
+    <mergeCell ref="F113:F114"/>
+    <mergeCell ref="G113:G114"/>
+    <mergeCell ref="H113:H114"/>
+    <mergeCell ref="I113:I114"/>
+    <mergeCell ref="B124:C124"/>
+    <mergeCell ref="D124:E124"/>
+    <mergeCell ref="F124:G124"/>
+    <mergeCell ref="H124:I124"/>
+    <mergeCell ref="A125:A128"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="C126:C127"/>
+    <mergeCell ref="D126:D127"/>
+    <mergeCell ref="E126:E127"/>
+    <mergeCell ref="F126:F127"/>
+    <mergeCell ref="G126:G127"/>
+    <mergeCell ref="H126:H127"/>
+    <mergeCell ref="I126:I127"/>
+    <mergeCell ref="J141:K141"/>
+    <mergeCell ref="A150:A151"/>
+    <mergeCell ref="B150:C150"/>
+    <mergeCell ref="D150:E150"/>
+    <mergeCell ref="F150:G150"/>
+    <mergeCell ref="H150:I150"/>
+    <mergeCell ref="J150:K150"/>
+    <mergeCell ref="A141:A142"/>
+    <mergeCell ref="B141:C141"/>
+    <mergeCell ref="D141:E141"/>
+    <mergeCell ref="F141:G141"/>
+    <mergeCell ref="H141:I141"/>
+    <mergeCell ref="B160:C160"/>
+    <mergeCell ref="D160:E160"/>
+    <mergeCell ref="F160:G160"/>
+    <mergeCell ref="H160:I160"/>
+    <mergeCell ref="A161:A164"/>
+    <mergeCell ref="B162:B163"/>
+    <mergeCell ref="C162:C163"/>
+    <mergeCell ref="D162:D163"/>
+    <mergeCell ref="E162:E163"/>
+    <mergeCell ref="F162:F163"/>
+    <mergeCell ref="G162:G163"/>
+    <mergeCell ref="H162:H163"/>
+    <mergeCell ref="I162:I163"/>
+    <mergeCell ref="B173:C173"/>
+    <mergeCell ref="D173:E173"/>
+    <mergeCell ref="F173:G173"/>
+    <mergeCell ref="H173:I173"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="B175:B176"/>
+    <mergeCell ref="C175:C176"/>
+    <mergeCell ref="D175:D176"/>
+    <mergeCell ref="E175:E176"/>
+    <mergeCell ref="F175:F176"/>
+    <mergeCell ref="G175:G176"/>
+    <mergeCell ref="H175:H176"/>
+    <mergeCell ref="I175:I176"/>
+    <mergeCell ref="J189:K189"/>
+    <mergeCell ref="A195:A196"/>
+    <mergeCell ref="B195:C195"/>
+    <mergeCell ref="D195:E195"/>
+    <mergeCell ref="F195:G195"/>
+    <mergeCell ref="H195:I195"/>
+    <mergeCell ref="J195:K195"/>
+    <mergeCell ref="A189:A190"/>
+    <mergeCell ref="B189:C189"/>
+    <mergeCell ref="D189:E189"/>
+    <mergeCell ref="F189:G189"/>
+    <mergeCell ref="H189:I189"/>
+    <mergeCell ref="A218:A219"/>
+    <mergeCell ref="B218:C218"/>
+    <mergeCell ref="D218:E218"/>
+    <mergeCell ref="F218:G218"/>
+    <mergeCell ref="H218:I218"/>
+    <mergeCell ref="J218:K218"/>
+    <mergeCell ref="A203:A204"/>
+    <mergeCell ref="B203:C203"/>
+    <mergeCell ref="D203:E203"/>
+    <mergeCell ref="F203:G203"/>
+    <mergeCell ref="H203:I203"/>
+    <mergeCell ref="J203:K203"/>
     <mergeCell ref="A211:A212"/>
     <mergeCell ref="B211:C211"/>
     <mergeCell ref="D211:E211"/>
     <mergeCell ref="F211:G211"/>
     <mergeCell ref="H211:I211"/>
     <mergeCell ref="J211:K211"/>
-    <mergeCell ref="J67:K67"/>
-    <mergeCell ref="A67:A68"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="H67:I67"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="J76:K76"/>
-    <mergeCell ref="A76:A77"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="A85:A88"/>
-    <mergeCell ref="B86:B87"/>
-    <mergeCell ref="C86:C87"/>
-    <mergeCell ref="D86:D87"/>
-    <mergeCell ref="E86:E87"/>
-    <mergeCell ref="F86:F87"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>